<commit_message>
covnerted visio files to readable PDF files.
</commit_message>
<xml_diff>
--- a/Metrics/TimeGraphs.xlsx
+++ b/Metrics/TimeGraphs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Metrics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Desktop\2026 Y3 BIT\trimester2\Capstone\BHB-Capstone\Metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9B12405A-E811-4AF6-99FE-4D99CF93FFE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30E61C2F-FEA3-4524-8348-A6E8F93C973E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28ACBA2-C292-4647-A5A9-0895D9ED674B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4290" yWindow="4560" windowWidth="21600" windowHeight="11385" tabRatio="846" activeTab="1" xr2:uid="{72DB8043-9B22-441A-BCD0-4EB4CA42FDB6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="846" activeTab="1" xr2:uid="{72DB8043-9B22-441A-BCD0-4EB4CA42FDB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Human vs AI v1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="20">
   <si>
     <t>NMAP</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>Average</t>
+  </si>
+  <si>
+    <t>Wireshark Script Creation time</t>
+  </si>
+  <si>
+    <t>Human</t>
   </si>
 </sst>
 </file>
@@ -1207,6 +1213,2459 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1212007888"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-NZ"/>
+              <a:t>FOREMOST - HUMAN vs AI (Seconds)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="5.7137865923366428E-2"/>
+          <c:y val="0.18303258967629046"/>
+          <c:w val="0.93125329154410352"/>
+          <c:h val="0.70993839311752693"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Human vs AI v2'!$L$2:$L$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>FOREMOST</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>HUMAN</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Human vs AI v2'!$H$5:$H$17</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Eight.dd </c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Nine.dd</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Three.dd</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>AI</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Eight.dd </c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nine.dd</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Three.dd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Human vs AI v2'!$L$5:$L$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>14400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>77400</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10800</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>45</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-ED92-46B8-B638-00F855E4F8C4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1666216544"/>
+        <c:axId val="1010493968"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$I$2:$I$4</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="3"/>
+                      <c:pt idx="0">
+                        <c:v>FOREMOST</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="tx1">
+                              <a:lumMod val="75000"/>
+                              <a:lumOff val="25000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="en-US"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="outEnd"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst>
+                    <c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1">
+                                <a:lumMod val="35000"/>
+                                <a:lumOff val="65000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                            <a:round/>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$H$5:$H$17</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="12"/>
+                      <c:pt idx="0">
+                        <c:v>Eight.dd </c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Nine.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Three.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>Eight.dd </c:v>
+                      </c:pt>
+                      <c:pt idx="10">
+                        <c:v>Nine.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>Three.dd</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$I$5:$I$17</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="13"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-ED92-46B8-B638-00F855E4F8C4}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$J$2:$J$4</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="3"/>
+                      <c:pt idx="0">
+                        <c:v>FOREMOST</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:solidFill>
+                    <a:schemeClr val="accent2"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="tx1">
+                              <a:lumMod val="75000"/>
+                              <a:lumOff val="25000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="en-US"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="outEnd"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                    <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1">
+                                <a:lumMod val="35000"/>
+                                <a:lumOff val="65000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                            <a:round/>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$H$5:$H$17</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="12"/>
+                      <c:pt idx="0">
+                        <c:v>Eight.dd </c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Nine.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Three.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>Eight.dd </c:v>
+                      </c:pt>
+                      <c:pt idx="10">
+                        <c:v>Nine.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>Three.dd</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$J$5:$J$17</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="13"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-ED92-46B8-B638-00F855E4F8C4}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$K$2:$K$4</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="3"/>
+                      <c:pt idx="0">
+                        <c:v>FOREMOST</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:solidFill>
+                    <a:schemeClr val="accent3"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="tx1">
+                              <a:lumMod val="75000"/>
+                              <a:lumOff val="25000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="en-US"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="outEnd"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                    <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1">
+                                <a:lumMod val="35000"/>
+                                <a:lumOff val="65000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                            <a:round/>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$H$5:$H$17</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="12"/>
+                      <c:pt idx="0">
+                        <c:v>Eight.dd </c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Nine.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Three.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>Eight.dd </c:v>
+                      </c:pt>
+                      <c:pt idx="10">
+                        <c:v>Nine.dd</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>Three.dd</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$K$5:$K$17</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="13"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000003-ED92-46B8-B638-00F855E4F8C4}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+          </c:ext>
+        </c:extLst>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1666216544"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1010493968"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1010493968"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1666216544"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Human vs AI v2'!$F$54:$F$56</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>WIRESHARK</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>HUMAN</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent4">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent4">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Human vs AI v2'!$B$58:$B$68</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Evidence01.pcap</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Evidence02.pcap</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Evidence03.pcap</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>AI</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Wireshark Script Creation time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Human vs AI v2'!$F$58:$F$68</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.15</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>168</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-C9C3-4E69-BCFE-9B67D8033BE5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="115"/>
+        <c:overlap val="-20"/>
+        <c:axId val="1251188400"/>
+        <c:axId val="1251411696"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$C$54:$C$56</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="3"/>
+                      <c:pt idx="0">
+                        <c:v>WIRESHARK</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:gradFill rotWithShape="1">
+                    <a:gsLst>
+                      <a:gs pos="0">
+                        <a:schemeClr val="accent1">
+                          <a:satMod val="103000"/>
+                          <a:lumMod val="102000"/>
+                          <a:tint val="94000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="50000">
+                        <a:schemeClr val="accent1">
+                          <a:satMod val="110000"/>
+                          <a:lumMod val="100000"/>
+                          <a:shade val="100000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="100000">
+                        <a:schemeClr val="accent1">
+                          <a:lumMod val="99000"/>
+                          <a:satMod val="120000"/>
+                          <a:shade val="78000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                    </a:gsLst>
+                    <a:lin ang="5400000" scaled="0"/>
+                  </a:gradFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$B$58:$B$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="9"/>
+                      <c:pt idx="0">
+                        <c:v>Evidence01.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Evidence02.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Evidence03.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>Wireshark Script Creation time</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$C$58:$C$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="11"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-C9C3-4E69-BCFE-9B67D8033BE5}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$D$54:$D$56</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="3"/>
+                      <c:pt idx="0">
+                        <c:v>WIRESHARK</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:gradFill rotWithShape="1">
+                    <a:gsLst>
+                      <a:gs pos="0">
+                        <a:schemeClr val="accent2">
+                          <a:satMod val="103000"/>
+                          <a:lumMod val="102000"/>
+                          <a:tint val="94000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="50000">
+                        <a:schemeClr val="accent2">
+                          <a:satMod val="110000"/>
+                          <a:lumMod val="100000"/>
+                          <a:shade val="100000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="100000">
+                        <a:schemeClr val="accent2">
+                          <a:lumMod val="99000"/>
+                          <a:satMod val="120000"/>
+                          <a:shade val="78000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                    </a:gsLst>
+                    <a:lin ang="5400000" scaled="0"/>
+                  </a:gradFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$B$58:$B$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="9"/>
+                      <c:pt idx="0">
+                        <c:v>Evidence01.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Evidence02.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Evidence03.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>Wireshark Script Creation time</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$D$58:$D$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="11"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-C9C3-4E69-BCFE-9B67D8033BE5}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$E$54:$E$56</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="3"/>
+                      <c:pt idx="0">
+                        <c:v>WIRESHARK</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:gradFill rotWithShape="1">
+                    <a:gsLst>
+                      <a:gs pos="0">
+                        <a:schemeClr val="accent3">
+                          <a:satMod val="103000"/>
+                          <a:lumMod val="102000"/>
+                          <a:tint val="94000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="50000">
+                        <a:schemeClr val="accent3">
+                          <a:satMod val="110000"/>
+                          <a:lumMod val="100000"/>
+                          <a:shade val="100000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="100000">
+                        <a:schemeClr val="accent3">
+                          <a:lumMod val="99000"/>
+                          <a:satMod val="120000"/>
+                          <a:shade val="78000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                    </a:gsLst>
+                    <a:lin ang="5400000" scaled="0"/>
+                  </a:gradFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$B$58:$B$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="9"/>
+                      <c:pt idx="0">
+                        <c:v>Evidence01.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Evidence02.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Evidence03.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>Wireshark Script Creation time</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$E$58:$E$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="11"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-C9C3-4E69-BCFE-9B67D8033BE5}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+          </c:ext>
+        </c:extLst>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1251188400"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1251411696"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1251411696"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1251188400"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Human vs AI v2'!$F$53:$F$56</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="1">
+                  <c:v>WIRESHARK</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>HUMAN</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent4">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent4">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="lt1">
+                        <a:lumMod val="85000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="95000"/>
+                          <a:alpha val="54000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Human vs AI v2'!$B$57:$B$68</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Human</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Evidence01.pcap</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Evidence02.pcap</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Evidence03.pcap</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>AI</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Wireshark Script Creation time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Human vs AI v2'!$F$57:$F$68</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.15</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>168</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-5E31-4E5E-8E23-A3B0C12CB380}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="100"/>
+        <c:overlap val="-24"/>
+        <c:axId val="1331706320"/>
+        <c:axId val="1251327216"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$C$53:$C$56</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="4"/>
+                      <c:pt idx="1">
+                        <c:v>WIRESHARK</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:gradFill rotWithShape="1">
+                    <a:gsLst>
+                      <a:gs pos="0">
+                        <a:schemeClr val="accent1">
+                          <a:satMod val="103000"/>
+                          <a:lumMod val="102000"/>
+                          <a:tint val="94000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="50000">
+                        <a:schemeClr val="accent1">
+                          <a:satMod val="110000"/>
+                          <a:lumMod val="100000"/>
+                          <a:shade val="100000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="100000">
+                        <a:schemeClr val="accent1">
+                          <a:lumMod val="99000"/>
+                          <a:satMod val="120000"/>
+                          <a:shade val="78000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                    </a:gsLst>
+                    <a:lin ang="5400000" scaled="0"/>
+                  </a:gradFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="lt1">
+                              <a:lumMod val="85000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="en-US"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="outEnd"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst>
+                    <c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525">
+                            <a:solidFill>
+                              <a:schemeClr val="lt1">
+                                <a:lumMod val="95000"/>
+                                <a:alpha val="54000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$B$57:$B$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>Human</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Evidence01.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Evidence02.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>Evidence03.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>Wireshark Script Creation time</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$C$57:$C$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="12"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-5E31-4E5E-8E23-A3B0C12CB380}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$D$53:$D$56</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="4"/>
+                      <c:pt idx="1">
+                        <c:v>WIRESHARK</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:gradFill rotWithShape="1">
+                    <a:gsLst>
+                      <a:gs pos="0">
+                        <a:schemeClr val="accent2">
+                          <a:satMod val="103000"/>
+                          <a:lumMod val="102000"/>
+                          <a:tint val="94000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="50000">
+                        <a:schemeClr val="accent2">
+                          <a:satMod val="110000"/>
+                          <a:lumMod val="100000"/>
+                          <a:shade val="100000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="100000">
+                        <a:schemeClr val="accent2">
+                          <a:lumMod val="99000"/>
+                          <a:satMod val="120000"/>
+                          <a:shade val="78000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                    </a:gsLst>
+                    <a:lin ang="5400000" scaled="0"/>
+                  </a:gradFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="lt1">
+                              <a:lumMod val="85000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="en-US"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="outEnd"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst>
+                    <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525">
+                            <a:solidFill>
+                              <a:schemeClr val="lt1">
+                                <a:lumMod val="95000"/>
+                                <a:alpha val="54000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$B$57:$B$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>Human</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Evidence01.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Evidence02.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>Evidence03.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>Wireshark Script Creation time</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$D$57:$D$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="12"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-5E31-4E5E-8E23-A3B0C12CB380}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$E$53:$E$56</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="4"/>
+                      <c:pt idx="1">
+                        <c:v>WIRESHARK</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>HUMAN</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:gradFill rotWithShape="1">
+                    <a:gsLst>
+                      <a:gs pos="0">
+                        <a:schemeClr val="accent3">
+                          <a:satMod val="103000"/>
+                          <a:lumMod val="102000"/>
+                          <a:tint val="94000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="50000">
+                        <a:schemeClr val="accent3">
+                          <a:satMod val="110000"/>
+                          <a:lumMod val="100000"/>
+                          <a:shade val="100000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                      <a:gs pos="100000">
+                        <a:schemeClr val="accent3">
+                          <a:lumMod val="99000"/>
+                          <a:satMod val="120000"/>
+                          <a:shade val="78000"/>
+                        </a:schemeClr>
+                      </a:gs>
+                    </a:gsLst>
+                    <a:lin ang="5400000" scaled="0"/>
+                  </a:gradFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:dLbls>
+                  <c:spPr>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                  <c:txPr>
+                    <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                      <a:spAutoFit/>
+                    </a:bodyPr>
+                    <a:lstStyle/>
+                    <a:p>
+                      <a:pPr>
+                        <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                          <a:solidFill>
+                            <a:schemeClr val="lt1">
+                              <a:lumMod val="85000"/>
+                            </a:schemeClr>
+                          </a:solidFill>
+                          <a:latin typeface="+mn-lt"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
+                        </a:defRPr>
+                      </a:pPr>
+                      <a:endParaRPr lang="en-US"/>
+                    </a:p>
+                  </c:txPr>
+                  <c:dLblPos val="outEnd"/>
+                  <c:showLegendKey val="0"/>
+                  <c:showVal val="1"/>
+                  <c:showCatName val="0"/>
+                  <c:showSerName val="0"/>
+                  <c:showPercent val="0"/>
+                  <c:showBubbleSize val="0"/>
+                  <c:showLeaderLines val="0"/>
+                  <c:extLst>
+                    <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                      <c15:showLeaderLines val="1"/>
+                      <c15:leaderLines>
+                        <c:spPr>
+                          <a:ln w="9525">
+                            <a:solidFill>
+                              <a:schemeClr val="lt1">
+                                <a:lumMod val="95000"/>
+                                <a:alpha val="54000"/>
+                              </a:schemeClr>
+                            </a:solidFill>
+                          </a:ln>
+                          <a:effectLst/>
+                        </c:spPr>
+                      </c15:leaderLines>
+                    </c:ext>
+                  </c:extLst>
+                </c:dLbls>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$B$57:$B$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="10"/>
+                      <c:pt idx="0">
+                        <c:v>Human</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>Evidence01.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>Evidence02.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>Evidence03.pcap</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>AI</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>Wireshark Script Creation time</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Human vs AI v2'!$E$57:$E$68</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="12"/>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-5E31-4E5E-8E23-A3B0C12CB380}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+          </c:ext>
+        </c:extLst>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1331706320"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1251327216"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1251327216"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1331706320"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8430,6 +10889,9 @@
                 <c:pt idx="0">
                   <c:v>14400</c:v>
                 </c:pt>
+                <c:pt idx="1">
+                  <c:v>68400</c:v>
+                </c:pt>
                 <c:pt idx="2">
                   <c:v>25740</c:v>
                 </c:pt>
@@ -9159,6 +11621,126 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors12.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -10014,6 +12596,1501 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="222">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="34925" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style12.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="34925" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
   <cs:axisTitle>
@@ -14315,6 +18392,116 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{800DCEC6-B92B-415A-B104-83DEDD6E2BED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304799</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>128586</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>1847850</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF709C50-7413-B9B9-B2BF-B7D25907CDEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>1866900</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{257F0B83-6AE4-8FB8-BF89-B30E98DF8097}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16423,7 +20610,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6E417AB-164F-441C-A77F-D7440DFB6AE1}">
-  <dimension ref="A1:T18"/>
+  <dimension ref="A1:T122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -16592,7 +20779,9 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
+      <c r="R6" s="1">
+        <v>68400</v>
+      </c>
       <c r="S6" s="2"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -16901,6 +21090,585 @@
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
     </row>
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B54" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+    </row>
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B56" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="8"/>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B57" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B58" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B59" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B60" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1">
+        <v>7.15</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B61" s="10"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2"/>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B65" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="8"/>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B66" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+    </row>
+    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A106" s="2"/>
+      <c r="B106" s="2"/>
+      <c r="C106" s="2"/>
+      <c r="D106" s="2"/>
+      <c r="E106" s="2"/>
+      <c r="F106" s="2"/>
+      <c r="G106" s="2"/>
+      <c r="H106" s="2"/>
+      <c r="I106" s="2"/>
+      <c r="J106" s="2"/>
+      <c r="K106" s="2"/>
+      <c r="L106" s="2"/>
+      <c r="M106" s="2"/>
+      <c r="N106" s="2"/>
+      <c r="O106" s="2"/>
+      <c r="P106" s="2"/>
+      <c r="Q106" s="2"/>
+      <c r="R106" s="2"/>
+      <c r="S106" s="2"/>
+    </row>
+    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A107" s="2"/>
+      <c r="B107" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C107" s="2"/>
+      <c r="D107" s="2"/>
+      <c r="E107" s="2"/>
+      <c r="F107" s="2"/>
+      <c r="G107" s="2"/>
+      <c r="H107" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I107" s="2"/>
+      <c r="J107" s="2"/>
+      <c r="K107" s="2"/>
+      <c r="L107" s="2"/>
+      <c r="M107" s="2"/>
+      <c r="N107" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="O107" s="2"/>
+      <c r="P107" s="2"/>
+      <c r="Q107" s="2"/>
+      <c r="R107" s="2"/>
+      <c r="S107" s="2"/>
+    </row>
+    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A108" s="2"/>
+      <c r="B108" s="2"/>
+      <c r="C108" s="2"/>
+      <c r="D108" s="2"/>
+      <c r="E108" s="2"/>
+      <c r="F108" s="2"/>
+      <c r="G108" s="2"/>
+      <c r="H108" s="2"/>
+      <c r="I108" s="2"/>
+      <c r="J108" s="2"/>
+      <c r="K108" s="2"/>
+      <c r="L108" s="2"/>
+      <c r="M108" s="2"/>
+      <c r="N108" s="2"/>
+      <c r="O108" s="2"/>
+      <c r="P108" s="2"/>
+      <c r="Q108" s="2"/>
+      <c r="R108" s="2"/>
+      <c r="S108" s="2"/>
+    </row>
+    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A109" s="2"/>
+      <c r="B109" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3"/>
+      <c r="E109" s="3"/>
+      <c r="F109" s="8"/>
+      <c r="G109" s="2"/>
+      <c r="H109" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I109" s="3"/>
+      <c r="J109" s="3"/>
+      <c r="K109" s="3"/>
+      <c r="L109" s="8"/>
+      <c r="M109" s="2"/>
+      <c r="N109" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="O109" s="3"/>
+      <c r="P109" s="3"/>
+      <c r="Q109" s="3"/>
+      <c r="R109" s="8"/>
+      <c r="S109" s="2"/>
+    </row>
+    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A110" s="2"/>
+      <c r="B110" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="1">
+        <v>28800</v>
+      </c>
+      <c r="G110" s="2"/>
+      <c r="H110" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I110" s="1"/>
+      <c r="J110" s="1"/>
+      <c r="K110" s="1"/>
+      <c r="L110" s="1">
+        <v>14400</v>
+      </c>
+      <c r="M110" s="2"/>
+      <c r="N110" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O110" s="1"/>
+      <c r="P110" s="1"/>
+      <c r="Q110" s="1"/>
+      <c r="R110" s="1">
+        <v>14400</v>
+      </c>
+      <c r="S110" s="2"/>
+    </row>
+    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A111" s="2"/>
+      <c r="B111" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C111" s="1"/>
+      <c r="D111" s="1"/>
+      <c r="E111" s="1"/>
+      <c r="F111" s="1">
+        <v>19620</v>
+      </c>
+      <c r="G111" s="2"/>
+      <c r="H111" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I111" s="1"/>
+      <c r="J111" s="1"/>
+      <c r="K111" s="1"/>
+      <c r="L111" s="1">
+        <v>77400</v>
+      </c>
+      <c r="M111" s="2"/>
+      <c r="N111" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O111" s="1"/>
+      <c r="P111" s="1"/>
+      <c r="Q111" s="1"/>
+      <c r="R111" s="1">
+        <v>68400</v>
+      </c>
+      <c r="S111" s="2"/>
+    </row>
+    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A112" s="2"/>
+      <c r="B112" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C112" s="1"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+      <c r="F112" s="1">
+        <v>7200</v>
+      </c>
+      <c r="G112" s="2"/>
+      <c r="H112" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I112" s="1"/>
+      <c r="J112" s="1"/>
+      <c r="K112" s="1"/>
+      <c r="L112" s="1">
+        <v>10800</v>
+      </c>
+      <c r="M112" s="2"/>
+      <c r="N112" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O112" s="1"/>
+      <c r="P112" s="1"/>
+      <c r="Q112" s="1"/>
+      <c r="R112" s="1">
+        <v>25740</v>
+      </c>
+      <c r="S112" s="2"/>
+    </row>
+    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A113" s="2"/>
+      <c r="B113" s="10"/>
+      <c r="C113" s="2"/>
+      <c r="D113" s="2"/>
+      <c r="E113" s="2"/>
+      <c r="F113" s="2"/>
+      <c r="G113" s="2"/>
+      <c r="H113" s="10"/>
+      <c r="I113" s="2"/>
+      <c r="J113" s="2"/>
+      <c r="K113" s="2"/>
+      <c r="L113" s="2"/>
+      <c r="M113" s="2"/>
+      <c r="N113" s="10"/>
+      <c r="O113" s="2"/>
+      <c r="P113" s="2"/>
+      <c r="Q113" s="2"/>
+      <c r="R113" s="2"/>
+      <c r="S113" s="2"/>
+    </row>
+    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A114" s="2"/>
+      <c r="B114" s="2"/>
+      <c r="C114" s="2"/>
+      <c r="D114" s="2"/>
+      <c r="E114" s="2"/>
+      <c r="F114" s="2"/>
+      <c r="G114" s="2"/>
+      <c r="H114" s="2"/>
+      <c r="I114" s="2"/>
+      <c r="J114" s="2"/>
+      <c r="K114" s="2"/>
+      <c r="L114" s="2"/>
+      <c r="M114" s="2"/>
+      <c r="N114" s="2"/>
+      <c r="O114" s="2"/>
+      <c r="P114" s="2"/>
+      <c r="Q114" s="2"/>
+      <c r="R114" s="2"/>
+      <c r="S114" s="2"/>
+    </row>
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A115" s="2"/>
+      <c r="B115" s="2"/>
+      <c r="C115" s="2"/>
+      <c r="D115" s="2"/>
+      <c r="E115" s="2"/>
+      <c r="F115" s="2"/>
+      <c r="G115" s="2"/>
+      <c r="H115" s="2"/>
+      <c r="I115" s="2"/>
+      <c r="J115" s="2"/>
+      <c r="K115" s="2"/>
+      <c r="L115" s="2"/>
+      <c r="M115" s="2"/>
+      <c r="N115" s="2"/>
+      <c r="O115" s="2"/>
+      <c r="P115" s="2"/>
+      <c r="Q115" s="2"/>
+      <c r="R115" s="2"/>
+      <c r="S115" s="2"/>
+    </row>
+    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A116" s="2"/>
+      <c r="B116" s="2"/>
+      <c r="C116" s="2"/>
+      <c r="D116" s="2"/>
+      <c r="E116" s="2"/>
+      <c r="F116" s="2"/>
+      <c r="G116" s="2"/>
+      <c r="H116" s="2"/>
+      <c r="I116" s="2"/>
+      <c r="J116" s="2"/>
+      <c r="K116" s="2"/>
+      <c r="L116" s="2"/>
+      <c r="M116" s="2"/>
+      <c r="N116" s="2"/>
+      <c r="O116" s="2"/>
+      <c r="P116" s="2"/>
+      <c r="Q116" s="2"/>
+      <c r="R116" s="2"/>
+      <c r="S116" s="2"/>
+    </row>
+    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A117" s="2"/>
+      <c r="B117" s="2"/>
+      <c r="C117" s="2"/>
+      <c r="D117" s="2"/>
+      <c r="E117" s="2"/>
+      <c r="F117" s="2"/>
+      <c r="G117" s="2"/>
+      <c r="H117" s="2"/>
+      <c r="I117" s="2"/>
+      <c r="J117" s="2"/>
+      <c r="K117" s="2"/>
+      <c r="L117" s="2"/>
+      <c r="M117" s="2"/>
+      <c r="N117" s="2"/>
+      <c r="O117" s="2"/>
+      <c r="P117" s="2"/>
+      <c r="Q117" s="2"/>
+      <c r="R117" s="2"/>
+      <c r="S117" s="2"/>
+    </row>
+    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A118" s="2"/>
+      <c r="B118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="3"/>
+      <c r="D118" s="3"/>
+      <c r="E118" s="3"/>
+      <c r="F118" s="8"/>
+      <c r="G118" s="2"/>
+      <c r="H118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I118" s="3"/>
+      <c r="J118" s="3"/>
+      <c r="K118" s="3"/>
+      <c r="L118" s="8"/>
+      <c r="M118" s="2"/>
+      <c r="N118" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="O118" s="3"/>
+      <c r="P118" s="3"/>
+      <c r="Q118" s="3"/>
+      <c r="R118" s="8"/>
+      <c r="S118" s="2"/>
+    </row>
+    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A119" s="2"/>
+      <c r="B119" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C119" s="1"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="1"/>
+      <c r="F119" s="1">
+        <v>103</v>
+      </c>
+      <c r="G119" s="2"/>
+      <c r="H119" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I119" s="1"/>
+      <c r="J119" s="1"/>
+      <c r="K119" s="1"/>
+      <c r="L119" s="1">
+        <v>19</v>
+      </c>
+      <c r="M119" s="2"/>
+      <c r="N119" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O119" s="1"/>
+      <c r="P119" s="1"/>
+      <c r="Q119" s="1"/>
+      <c r="R119" s="1">
+        <v>157</v>
+      </c>
+      <c r="S119" s="2"/>
+    </row>
+    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A120" s="2"/>
+      <c r="B120" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C120" s="1"/>
+      <c r="D120" s="1"/>
+      <c r="E120" s="1"/>
+      <c r="F120" s="1">
+        <v>81</v>
+      </c>
+      <c r="G120" s="2"/>
+      <c r="H120" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I120" s="1"/>
+      <c r="J120" s="1"/>
+      <c r="K120" s="1"/>
+      <c r="L120" s="1">
+        <v>37</v>
+      </c>
+      <c r="M120" s="2"/>
+      <c r="N120" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O120" s="1"/>
+      <c r="P120" s="1"/>
+      <c r="Q120" s="1"/>
+      <c r="R120" s="1">
+        <v>115</v>
+      </c>
+      <c r="S120" s="2"/>
+    </row>
+    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A121" s="2"/>
+      <c r="B121" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C121" s="1"/>
+      <c r="D121" s="1"/>
+      <c r="E121" s="1"/>
+      <c r="F121" s="1">
+        <v>99</v>
+      </c>
+      <c r="G121" s="2"/>
+      <c r="H121" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I121" s="1"/>
+      <c r="J121" s="1"/>
+      <c r="K121" s="1"/>
+      <c r="L121" s="1">
+        <v>45</v>
+      </c>
+      <c r="M121" s="2"/>
+      <c r="N121" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O121" s="1"/>
+      <c r="P121" s="1"/>
+      <c r="Q121" s="1"/>
+      <c r="R121" s="1">
+        <v>137</v>
+      </c>
+      <c r="S121" s="2"/>
+    </row>
+    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A122" s="2"/>
+      <c r="B122" s="10"/>
+      <c r="C122" s="2"/>
+      <c r="D122" s="2"/>
+      <c r="E122" s="2"/>
+      <c r="F122" s="2"/>
+      <c r="G122" s="2"/>
+      <c r="H122" s="10"/>
+      <c r="I122" s="2"/>
+      <c r="J122" s="2"/>
+      <c r="K122" s="2"/>
+      <c r="L122" s="2"/>
+      <c r="M122" s="2"/>
+      <c r="N122" s="10"/>
+      <c r="O122" s="2"/>
+      <c r="P122" s="2"/>
+      <c r="Q122" s="2"/>
+      <c r="R122" s="2"/>
+      <c r="S122" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>